<commit_message>
New Episode of Lanterns, and Doctor Who Down for Maintenance
</commit_message>
<xml_diff>
--- a/DCU.xlsx
+++ b/DCU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05CA6065-87EC-4F4D-AAB2-CFDA6154C7FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7CBFB99-17ED-41FC-8718-0BAC4FBF7FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21697" yWindow="-1140" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="21720" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DCUDATASHEET" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="410">
   <si>
     <t>id</t>
   </si>
@@ -1211,9 +1211,6 @@
     <t>Fall, 2016</t>
   </si>
   <si>
-    <t>Winter, 2026</t>
-  </si>
-  <si>
     <t>June, 2016</t>
   </si>
   <si>
@@ -1235,9 +1232,6 @@
     <t>September, 2026</t>
   </si>
   <si>
-    <t>Episode 1</t>
-  </si>
-  <si>
     <t>November, 1918</t>
   </si>
   <si>
@@ -1266,6 +1260,12 @@
   </si>
   <si>
     <t>February, 2020</t>
+  </si>
+  <si>
+    <t>Trust Fall</t>
+  </si>
+  <si>
+    <t>Pilot</t>
   </si>
 </sst>
 </file>
@@ -1744,10 +1744,10 @@
         <v>42888</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="K2" t="s">
         <v>18</v>
@@ -1791,10 +1791,10 @@
         <v>42997</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="K3" t="s">
         <v>18</v>
@@ -2043,10 +2043,10 @@
         <v>44181</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K9" t="s">
         <v>18</v>
@@ -2418,10 +2418,10 @@
         <v>41439</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="K18" t="s">
         <v>18</v>
@@ -2465,10 +2465,10 @@
         <v>42454</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K19" t="s">
         <v>18</v>
@@ -2512,10 +2512,10 @@
         <v>42587</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="K20" t="s">
         <v>18</v>
@@ -2556,7 +2556,7 @@
         <v>122</v>
       </c>
       <c r="F21" t="s">
-        <v>399</v>
+        <v>409</v>
       </c>
       <c r="H21" s="1">
         <v>46250</v>
@@ -2565,7 +2565,7 @@
         <v>390</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="K21" t="s">
         <v>196</v>
@@ -2588,93 +2588,93 @@
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>248</v>
       </c>
       <c r="B22">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="C22">
-        <v>21</v>
+        <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>100</v>
-      </c>
-      <c r="G22">
-        <v>242</v>
+        <v>245</v>
+      </c>
+      <c r="E22" t="s">
+        <v>129</v>
+      </c>
+      <c r="F22" t="s">
+        <v>408</v>
       </c>
       <c r="H22" s="1">
-        <v>43056</v>
+        <v>46257</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>406</v>
+        <v>390</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>406</v>
+        <v>390</v>
       </c>
       <c r="K22" t="s">
-        <v>18</v>
+        <v>196</v>
       </c>
       <c r="M22" t="s">
-        <v>101</v>
+        <v>246</v>
       </c>
       <c r="N22" t="s">
-        <v>20</v>
-      </c>
-      <c r="O22" t="s">
-        <v>282</v>
+        <v>125</v>
       </c>
       <c r="P22" t="s">
-        <v>307</v>
+        <v>355</v>
       </c>
       <c r="Q22" t="s">
-        <v>102</v>
+        <v>247</v>
       </c>
       <c r="R22" t="s">
-        <v>22</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B23">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C23">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="G23">
-        <v>143</v>
+        <v>242</v>
       </c>
       <c r="H23" s="1">
-        <v>43455</v>
+        <v>43056</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>393</v>
+        <v>404</v>
       </c>
       <c r="K23" t="s">
         <v>18</v>
       </c>
       <c r="M23" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="N23" t="s">
         <v>20</v>
       </c>
       <c r="O23" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="P23" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="Q23" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="R23" t="s">
         <v>22</v>
@@ -2682,46 +2682,46 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B24">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C24">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D24" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G24">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="H24" s="1">
-        <v>43560</v>
+        <v>43455</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>408</v>
+        <v>392</v>
       </c>
       <c r="K24" t="s">
         <v>18</v>
       </c>
       <c r="M24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="N24" t="s">
         <v>20</v>
       </c>
       <c r="O24" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="P24" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Q24" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="R24" t="s">
         <v>22</v>
@@ -2729,46 +2729,46 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B25">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C25">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D25" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G25">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="H25" s="1">
-        <v>43868</v>
+        <v>43560</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="K25" t="s">
         <v>18</v>
       </c>
       <c r="M25" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="N25" t="s">
         <v>20</v>
       </c>
       <c r="O25" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="P25" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="Q25" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="R25" t="s">
         <v>22</v>
@@ -2776,46 +2776,46 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B26">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C26">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D26" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G26">
-        <v>132</v>
+        <v>109</v>
       </c>
       <c r="H26" s="1">
-        <v>44407</v>
+        <v>43868</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>395</v>
+        <v>407</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>395</v>
+        <v>407</v>
       </c>
       <c r="K26" t="s">
-        <v>117</v>
+        <v>18</v>
       </c>
       <c r="M26" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="N26" t="s">
         <v>20</v>
       </c>
       <c r="O26" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="P26" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="Q26" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="R26" t="s">
         <v>22</v>
@@ -2823,84 +2823,81 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B27">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C27">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D27" t="s">
-        <v>121</v>
-      </c>
-      <c r="E27" t="s">
-        <v>122</v>
-      </c>
-      <c r="F27" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="G27">
-        <v>46</v>
+        <v>132</v>
       </c>
       <c r="H27" s="1">
-        <v>44574</v>
+        <v>44407</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="K27" t="s">
         <v>117</v>
       </c>
       <c r="M27" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="N27" t="s">
-        <v>125</v>
+        <v>20</v>
+      </c>
+      <c r="O27" t="s">
+        <v>288</v>
       </c>
       <c r="P27" t="s">
-        <v>338</v>
+        <v>314</v>
       </c>
       <c r="Q27" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="R27" t="s">
-        <v>127</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B28">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C28">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D28" t="s">
         <v>121</v>
       </c>
       <c r="E28" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="F28" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="G28">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="H28" s="1">
         <v>44574</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="K28" t="s">
         <v>117</v>
@@ -2912,7 +2909,7 @@
         <v>125</v>
       </c>
       <c r="P28" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="Q28" t="s">
         <v>126</v>
@@ -2923,34 +2920,34 @@
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B29">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C29">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D29" t="s">
         <v>121</v>
       </c>
       <c r="E29" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F29" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="G29">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H29" s="1">
         <v>44574</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="K29" t="s">
         <v>117</v>
@@ -2962,7 +2959,7 @@
         <v>125</v>
       </c>
       <c r="P29" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="Q29" t="s">
         <v>126</v>
@@ -2973,34 +2970,34 @@
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B30">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C30">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D30" t="s">
         <v>121</v>
       </c>
       <c r="E30" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F30" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G30">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="H30" s="1">
-        <v>44581</v>
+        <v>44574</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="K30" t="s">
         <v>117</v>
@@ -3012,7 +3009,7 @@
         <v>125</v>
       </c>
       <c r="P30" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="Q30" t="s">
         <v>126</v>
@@ -3023,34 +3020,34 @@
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B31">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C31">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D31" t="s">
         <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F31" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G31">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H31" s="1">
-        <v>44588</v>
+        <v>44581</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="K31" t="s">
         <v>117</v>
@@ -3062,7 +3059,7 @@
         <v>125</v>
       </c>
       <c r="P31" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="Q31" t="s">
         <v>126</v>
@@ -3073,34 +3070,34 @@
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B32">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C32">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D32" t="s">
         <v>121</v>
       </c>
       <c r="E32" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F32" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="G32">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H32" s="1">
-        <v>44595</v>
+        <v>44588</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="K32" t="s">
         <v>117</v>
@@ -3112,7 +3109,7 @@
         <v>125</v>
       </c>
       <c r="P32" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="Q32" t="s">
         <v>126</v>
@@ -3123,34 +3120,34 @@
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B33">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C33">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D33" t="s">
         <v>121</v>
       </c>
       <c r="E33" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F33" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="G33">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="H33" s="1">
-        <v>44602</v>
+        <v>44595</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="K33" t="s">
         <v>117</v>
@@ -3162,7 +3159,7 @@
         <v>125</v>
       </c>
       <c r="P33" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="Q33" t="s">
         <v>126</v>
@@ -3173,34 +3170,34 @@
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B34">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C34">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D34" t="s">
         <v>121</v>
       </c>
       <c r="E34" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F34" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G34">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="H34" s="1">
-        <v>44609</v>
+        <v>44602</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="K34" t="s">
         <v>117</v>
@@ -3212,7 +3209,7 @@
         <v>125</v>
       </c>
       <c r="P34" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="Q34" t="s">
         <v>126</v>
@@ -3223,87 +3220,93 @@
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B35">
+        <v>31</v>
+      </c>
+      <c r="C35">
         <v>33</v>
       </c>
-      <c r="C35">
-        <v>34</v>
-      </c>
       <c r="D35" t="s">
-        <v>150</v>
+        <v>121</v>
+      </c>
+      <c r="E35" t="s">
+        <v>147</v>
+      </c>
+      <c r="F35" t="s">
+        <v>148</v>
+      </c>
+      <c r="G35">
+        <v>45</v>
       </c>
       <c r="H35" s="1">
-        <v>44855</v>
+        <v>44609</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="K35" t="s">
-        <v>18</v>
+        <v>117</v>
       </c>
       <c r="M35" t="s">
-        <v>151</v>
+        <v>124</v>
       </c>
       <c r="N35" t="s">
-        <v>20</v>
-      </c>
-      <c r="O35" t="s">
-        <v>290</v>
+        <v>125</v>
       </c>
       <c r="P35" t="s">
-        <v>312</v>
+        <v>345</v>
       </c>
       <c r="Q35" t="s">
-        <v>152</v>
+        <v>126</v>
       </c>
       <c r="R35" t="s">
-        <v>22</v>
+        <v>127</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B36">
+        <v>33</v>
+      </c>
+      <c r="C36">
         <v>34</v>
       </c>
-      <c r="C36">
-        <v>35</v>
-      </c>
       <c r="D36" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="H36" s="1">
-        <v>45002</v>
+        <v>44855</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="K36" t="s">
         <v>18</v>
       </c>
       <c r="M36" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="N36" t="s">
         <v>20</v>
       </c>
       <c r="O36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="P36" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="Q36" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="R36" t="s">
         <v>22</v>
@@ -3311,43 +3314,43 @@
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B37">
+        <v>34</v>
+      </c>
+      <c r="C37">
         <v>35</v>
       </c>
-      <c r="C37">
-        <v>36</v>
-      </c>
       <c r="D37" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="H37" s="1">
-        <v>45093</v>
+        <v>45002</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K37" t="s">
         <v>18</v>
       </c>
       <c r="M37" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="N37" t="s">
         <v>20</v>
       </c>
       <c r="O37" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="P37" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="Q37" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="R37" t="s">
         <v>22</v>
@@ -3355,43 +3358,43 @@
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B38">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C38">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D38" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="H38" s="1">
-        <v>44624</v>
+        <v>45093</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="K38" t="s">
-        <v>163</v>
+        <v>18</v>
       </c>
       <c r="M38" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="N38" t="s">
         <v>20</v>
       </c>
       <c r="O38" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="P38" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="Q38" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="R38" t="s">
         <v>22</v>
@@ -3399,75 +3402,72 @@
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="B39">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C39">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D39" t="s">
-        <v>167</v>
-      </c>
-      <c r="E39" t="s">
-        <v>122</v>
-      </c>
-      <c r="F39" t="s">
-        <v>168</v>
-      </c>
-      <c r="G39">
-        <v>67</v>
+        <v>162</v>
       </c>
       <c r="H39" s="1">
-        <v>45555</v>
+        <v>44624</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>383</v>
       </c>
       <c r="K39" t="s">
         <v>163</v>
       </c>
       <c r="M39" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="N39" t="s">
-        <v>125</v>
+        <v>20</v>
       </c>
       <c r="O39" t="s">
-        <v>302</v>
+        <v>289</v>
       </c>
       <c r="P39" t="s">
-        <v>362</v>
+        <v>311</v>
       </c>
       <c r="Q39" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="R39" t="s">
-        <v>127</v>
+        <v>22</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="B40">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C40">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D40" t="s">
         <v>167</v>
       </c>
       <c r="E40" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="F40" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G40">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="H40" s="1">
-        <v>45565</v>
+        <v>45555</v>
       </c>
       <c r="K40" t="s">
         <v>163</v>
@@ -3482,7 +3482,7 @@
         <v>302</v>
       </c>
       <c r="P40" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="Q40" t="s">
         <v>170</v>
@@ -3493,28 +3493,28 @@
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B41">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C41">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D41" t="s">
         <v>167</v>
       </c>
       <c r="E41" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F41" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G41">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H41" s="1">
-        <v>45572</v>
+        <v>45565</v>
       </c>
       <c r="K41" t="s">
         <v>163</v>
@@ -3529,7 +3529,7 @@
         <v>302</v>
       </c>
       <c r="P41" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="Q41" t="s">
         <v>170</v>
@@ -3540,28 +3540,28 @@
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B42">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C42">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D42" t="s">
         <v>167</v>
       </c>
       <c r="E42" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F42" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G42">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H42" s="1">
-        <v>45579</v>
+        <v>45572</v>
       </c>
       <c r="K42" t="s">
         <v>163</v>
@@ -3576,7 +3576,7 @@
         <v>302</v>
       </c>
       <c r="P42" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="Q42" t="s">
         <v>170</v>
@@ -3587,33 +3587,33 @@
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B43">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C43">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D43" t="s">
         <v>167</v>
       </c>
       <c r="E43" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F43" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="G43">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H43" s="1">
-        <v>45586</v>
+        <v>45579</v>
       </c>
       <c r="K43" t="s">
         <v>163</v>
       </c>
-      <c r="M43" s="2" t="s">
+      <c r="M43" t="s">
         <v>169</v>
       </c>
       <c r="N43" t="s">
@@ -3623,7 +3623,7 @@
         <v>302</v>
       </c>
       <c r="P43" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="Q43" t="s">
         <v>170</v>
@@ -3634,33 +3634,33 @@
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B44">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C44">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D44" t="s">
         <v>167</v>
       </c>
       <c r="E44" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F44" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G44">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H44" s="1">
-        <v>45593</v>
+        <v>45586</v>
       </c>
       <c r="K44" t="s">
         <v>163</v>
       </c>
-      <c r="M44" t="s">
+      <c r="M44" s="2" t="s">
         <v>169</v>
       </c>
       <c r="N44" t="s">
@@ -3670,7 +3670,7 @@
         <v>302</v>
       </c>
       <c r="P44" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="Q44" t="s">
         <v>170</v>
@@ -3681,28 +3681,28 @@
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B45">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C45">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D45" t="s">
         <v>167</v>
       </c>
       <c r="E45" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F45" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G45">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="H45" s="1">
-        <v>45600</v>
+        <v>45593</v>
       </c>
       <c r="K45" t="s">
         <v>163</v>
@@ -3717,7 +3717,7 @@
         <v>302</v>
       </c>
       <c r="P45" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="Q45" t="s">
         <v>170</v>
@@ -3728,28 +3728,28 @@
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B46">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C46">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D46" t="s">
         <v>167</v>
       </c>
       <c r="E46" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F46" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G46">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="H46" s="1">
-        <v>45607</v>
+        <v>45600</v>
       </c>
       <c r="K46" t="s">
         <v>163</v>
@@ -3764,7 +3764,7 @@
         <v>302</v>
       </c>
       <c r="P46" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="Q46" t="s">
         <v>170</v>
@@ -3775,87 +3775,90 @@
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B47">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C47">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D47" t="s">
-        <v>186</v>
+        <v>167</v>
+      </c>
+      <c r="E47" t="s">
+        <v>147</v>
+      </c>
+      <c r="F47" t="s">
+        <v>184</v>
+      </c>
+      <c r="G47">
+        <v>68</v>
       </c>
       <c r="H47" s="1">
-        <v>45282</v>
-      </c>
-      <c r="I47" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="J47" s="3" t="s">
-        <v>383</v>
+        <v>45607</v>
       </c>
       <c r="K47" t="s">
-        <v>18</v>
+        <v>163</v>
       </c>
       <c r="M47" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="N47" t="s">
-        <v>20</v>
+        <v>125</v>
       </c>
       <c r="O47" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="P47" t="s">
-        <v>317</v>
+        <v>369</v>
       </c>
       <c r="Q47" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="R47" t="s">
-        <v>22</v>
+        <v>127</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B48">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C48">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D48" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="H48" s="1">
-        <v>45156</v>
+        <v>45282</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>397</v>
+        <v>383</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="K48" t="s">
         <v>18</v>
       </c>
       <c r="M48" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="N48" t="s">
         <v>20</v>
       </c>
       <c r="O48" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="P48" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="Q48" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="R48" t="s">
         <v>22</v>
@@ -3863,75 +3866,69 @@
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B49">
+        <v>36</v>
+      </c>
+      <c r="C49">
         <v>47</v>
       </c>
-      <c r="C49">
-        <v>48</v>
-      </c>
       <c r="D49" t="s">
-        <v>194</v>
-      </c>
-      <c r="E49" t="s">
-        <v>122</v>
-      </c>
-      <c r="F49" t="s">
-        <v>195</v>
-      </c>
-      <c r="G49">
-        <v>23</v>
+        <v>190</v>
       </c>
       <c r="H49" s="1">
-        <v>45631</v>
+        <v>45156</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>379</v>
+        <v>396</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="K49" t="s">
-        <v>196</v>
+        <v>18</v>
       </c>
       <c r="M49" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="N49" t="s">
-        <v>125</v>
+        <v>20</v>
+      </c>
+      <c r="O49" t="s">
+        <v>294</v>
       </c>
       <c r="P49" t="s">
-        <v>370</v>
+        <v>318</v>
       </c>
       <c r="Q49" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="R49" t="s">
-        <v>127</v>
+        <v>22</v>
       </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B50">
+        <v>47</v>
+      </c>
+      <c r="C50">
         <v>48</v>
-      </c>
-      <c r="C50">
-        <v>49</v>
       </c>
       <c r="D50" t="s">
         <v>194</v>
       </c>
       <c r="E50" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="F50" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="G50">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H50" s="1">
         <v>45631</v>
@@ -3952,7 +3949,7 @@
         <v>125</v>
       </c>
       <c r="P50" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="Q50" t="s">
         <v>198</v>
@@ -3963,28 +3960,28 @@
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B51">
+        <v>48</v>
+      </c>
+      <c r="C51">
         <v>49</v>
-      </c>
-      <c r="C51">
-        <v>50</v>
       </c>
       <c r="D51" t="s">
         <v>194</v>
       </c>
       <c r="E51" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F51" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G51">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H51" s="1">
-        <v>45638</v>
+        <v>45631</v>
       </c>
       <c r="I51" s="3" t="s">
         <v>379</v>
@@ -4002,7 +3999,7 @@
         <v>125</v>
       </c>
       <c r="P51" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="Q51" t="s">
         <v>198</v>
@@ -4013,28 +4010,28 @@
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B52">
+        <v>49</v>
+      </c>
+      <c r="C52">
         <v>50</v>
-      </c>
-      <c r="C52">
-        <v>51</v>
       </c>
       <c r="D52" t="s">
         <v>194</v>
       </c>
       <c r="E52" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F52" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="G52">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H52" s="1">
-        <v>45645</v>
+        <v>45638</v>
       </c>
       <c r="I52" s="3" t="s">
         <v>379</v>
@@ -4052,7 +4049,7 @@
         <v>125</v>
       </c>
       <c r="P52" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="Q52" t="s">
         <v>198</v>
@@ -4063,28 +4060,28 @@
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B53">
+        <v>50</v>
+      </c>
+      <c r="C53">
         <v>51</v>
-      </c>
-      <c r="C53">
-        <v>52</v>
       </c>
       <c r="D53" t="s">
         <v>194</v>
       </c>
       <c r="E53" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F53" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G53">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H53" s="1">
-        <v>45652</v>
+        <v>45645</v>
       </c>
       <c r="I53" s="3" t="s">
         <v>379</v>
@@ -4102,7 +4099,7 @@
         <v>125</v>
       </c>
       <c r="P53" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="Q53" t="s">
         <v>198</v>
@@ -4113,28 +4110,28 @@
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B54">
+        <v>51</v>
+      </c>
+      <c r="C54">
         <v>52</v>
-      </c>
-      <c r="C54">
-        <v>53</v>
       </c>
       <c r="D54" t="s">
         <v>194</v>
       </c>
       <c r="E54" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F54" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G54">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H54" s="1">
-        <v>45659</v>
+        <v>45652</v>
       </c>
       <c r="I54" s="3" t="s">
         <v>379</v>
@@ -4152,7 +4149,7 @@
         <v>125</v>
       </c>
       <c r="P54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="Q54" t="s">
         <v>198</v>
@@ -4163,28 +4160,28 @@
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B55">
+        <v>52</v>
+      </c>
+      <c r="C55">
         <v>53</v>
-      </c>
-      <c r="C55">
-        <v>54</v>
       </c>
       <c r="D55" t="s">
         <v>194</v>
       </c>
       <c r="E55" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F55" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="G55">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H55" s="1">
-        <v>45666</v>
+        <v>45659</v>
       </c>
       <c r="I55" s="3" t="s">
         <v>379</v>
@@ -4202,7 +4199,7 @@
         <v>125</v>
       </c>
       <c r="P55" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="Q55" t="s">
         <v>198</v>
@@ -4213,128 +4210,128 @@
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B56">
+        <v>53</v>
+      </c>
+      <c r="C56">
         <v>54</v>
       </c>
-      <c r="C56">
-        <v>55</v>
-      </c>
       <c r="D56" t="s">
-        <v>29</v>
+        <v>194</v>
+      </c>
+      <c r="E56" t="s">
+        <v>144</v>
+      </c>
+      <c r="F56" t="s">
+        <v>210</v>
       </c>
       <c r="G56">
-        <v>129</v>
+        <v>27</v>
       </c>
       <c r="H56" s="1">
-        <v>45849</v>
-      </c>
-      <c r="I56" s="3">
-        <v>45796</v>
-      </c>
-      <c r="J56" s="3">
-        <v>45801</v>
+        <v>45666</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>379</v>
       </c>
       <c r="K56" t="s">
         <v>196</v>
       </c>
       <c r="M56" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="N56" t="s">
-        <v>20</v>
-      </c>
-      <c r="O56" t="s">
-        <v>296</v>
+        <v>125</v>
       </c>
       <c r="P56" t="s">
-        <v>315</v>
+        <v>376</v>
       </c>
       <c r="Q56" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="R56" t="s">
-        <v>22</v>
+        <v>127</v>
       </c>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B57">
+        <v>54</v>
+      </c>
+      <c r="C57">
         <v>55</v>
       </c>
-      <c r="C57">
-        <v>56</v>
-      </c>
       <c r="D57" t="s">
-        <v>121</v>
-      </c>
-      <c r="E57" t="s">
-        <v>215</v>
-      </c>
-      <c r="F57" t="s">
-        <v>216</v>
+        <v>29</v>
       </c>
       <c r="G57">
-        <v>44</v>
+        <v>129</v>
       </c>
       <c r="H57" s="1">
-        <v>45890</v>
-      </c>
-      <c r="I57" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="J57" s="3" t="s">
-        <v>380</v>
+        <v>45849</v>
+      </c>
+      <c r="I57" s="3">
+        <v>45796</v>
+      </c>
+      <c r="J57" s="3">
+        <v>45801</v>
       </c>
       <c r="K57" t="s">
         <v>196</v>
       </c>
       <c r="M57" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="N57" t="s">
-        <v>125</v>
+        <v>20</v>
+      </c>
+      <c r="O57" t="s">
+        <v>296</v>
       </c>
       <c r="P57" t="s">
-        <v>346</v>
+        <v>315</v>
       </c>
       <c r="Q57" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="R57" t="s">
-        <v>127</v>
+        <v>22</v>
       </c>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B58">
+        <v>55</v>
+      </c>
+      <c r="C58">
         <v>56</v>
-      </c>
-      <c r="C58">
-        <v>57</v>
       </c>
       <c r="D58" t="s">
         <v>121</v>
       </c>
       <c r="E58" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="F58" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="G58">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="H58" s="1">
-        <v>45897</v>
+        <v>45890</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="J58" s="3" t="s">
         <v>380</v>
@@ -4349,7 +4346,7 @@
         <v>125</v>
       </c>
       <c r="P58" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="Q58" t="s">
         <v>218</v>
@@ -4360,28 +4357,28 @@
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B59">
+        <v>56</v>
+      </c>
+      <c r="C59">
         <v>57</v>
-      </c>
-      <c r="C59">
-        <v>58</v>
       </c>
       <c r="D59" t="s">
         <v>121</v>
       </c>
       <c r="E59" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="F59" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="G59">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="H59" s="1">
-        <v>45904</v>
+        <v>45897</v>
       </c>
       <c r="I59" s="3" t="s">
         <v>380</v>
@@ -4399,7 +4396,7 @@
         <v>125</v>
       </c>
       <c r="P59" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="Q59" t="s">
         <v>218</v>
@@ -4410,28 +4407,28 @@
     </row>
     <row r="60" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B60">
+        <v>57</v>
+      </c>
+      <c r="C60">
         <v>58</v>
-      </c>
-      <c r="C60">
-        <v>59</v>
       </c>
       <c r="D60" t="s">
         <v>121</v>
       </c>
       <c r="E60" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F60" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G60">
         <v>39</v>
       </c>
       <c r="H60" s="1">
-        <v>45911</v>
+        <v>45904</v>
       </c>
       <c r="I60" s="3" t="s">
         <v>380</v>
@@ -4449,7 +4446,7 @@
         <v>125</v>
       </c>
       <c r="P60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="Q60" t="s">
         <v>218</v>
@@ -4460,28 +4457,28 @@
     </row>
     <row r="61" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B61">
+        <v>58</v>
+      </c>
+      <c r="C61">
         <v>59</v>
-      </c>
-      <c r="C61">
-        <v>60</v>
       </c>
       <c r="D61" t="s">
         <v>121</v>
       </c>
       <c r="E61" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F61" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="G61">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H61" s="1">
-        <v>45918</v>
+        <v>45911</v>
       </c>
       <c r="I61" s="3" t="s">
         <v>380</v>
@@ -4499,7 +4496,7 @@
         <v>125</v>
       </c>
       <c r="P61" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q61" t="s">
         <v>218</v>
@@ -4510,28 +4507,28 @@
     </row>
     <row r="62" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B62">
+        <v>59</v>
+      </c>
+      <c r="C62">
         <v>60</v>
-      </c>
-      <c r="C62">
-        <v>61</v>
       </c>
       <c r="D62" t="s">
         <v>121</v>
       </c>
       <c r="E62" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="F62" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="G62">
         <v>37</v>
       </c>
       <c r="H62" s="1">
-        <v>45925</v>
+        <v>45918</v>
       </c>
       <c r="I62" s="3" t="s">
         <v>380</v>
@@ -4549,7 +4546,7 @@
         <v>125</v>
       </c>
       <c r="P62" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Q62" t="s">
         <v>218</v>
@@ -4560,28 +4557,28 @@
     </row>
     <row r="63" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B63">
+        <v>60</v>
+      </c>
+      <c r="C63">
         <v>61</v>
-      </c>
-      <c r="C63">
-        <v>62</v>
       </c>
       <c r="D63" t="s">
         <v>121</v>
       </c>
       <c r="E63" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="F63" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="G63">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H63" s="1">
-        <v>45932</v>
+        <v>45925</v>
       </c>
       <c r="I63" s="3" t="s">
         <v>380</v>
@@ -4599,7 +4596,7 @@
         <v>125</v>
       </c>
       <c r="P63" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="Q63" t="s">
         <v>218</v>
@@ -4610,34 +4607,34 @@
     </row>
     <row r="64" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B64">
+        <v>61</v>
+      </c>
+      <c r="C64">
         <v>62</v>
-      </c>
-      <c r="C64">
-        <v>63</v>
       </c>
       <c r="D64" t="s">
         <v>121</v>
       </c>
       <c r="E64" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F64" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="G64">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="H64" s="1">
-        <v>45939</v>
+        <v>45932</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="K64" t="s">
         <v>196</v>
@@ -4649,7 +4646,7 @@
         <v>125</v>
       </c>
       <c r="P64" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="Q64" t="s">
         <v>218</v>
@@ -4660,87 +4657,99 @@
     </row>
     <row r="65" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B65">
+        <v>62</v>
+      </c>
+      <c r="C65">
         <v>63</v>
       </c>
-      <c r="C65">
-        <v>64</v>
-      </c>
       <c r="D65" t="s">
-        <v>241</v>
+        <v>121</v>
+      </c>
+      <c r="E65" t="s">
+        <v>238</v>
+      </c>
+      <c r="F65" t="s">
+        <v>239</v>
       </c>
       <c r="G65">
-        <v>107</v>
+        <v>58</v>
       </c>
       <c r="H65" s="1">
-        <v>46199</v>
+        <v>45939</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>398</v>
+        <v>381</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>398</v>
+        <v>381</v>
       </c>
       <c r="K65" t="s">
         <v>196</v>
       </c>
       <c r="M65" t="s">
-        <v>242</v>
+        <v>217</v>
       </c>
       <c r="N65" t="s">
-        <v>20</v>
-      </c>
-      <c r="O65" t="s">
-        <v>297</v>
+        <v>125</v>
       </c>
       <c r="P65" t="s">
-        <v>319</v>
+        <v>353</v>
       </c>
       <c r="Q65" t="s">
-        <v>243</v>
+        <v>218</v>
       </c>
       <c r="R65" t="s">
-        <v>22</v>
+        <v>127</v>
       </c>
     </row>
     <row r="66" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="B66">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C66">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D66" t="s">
-        <v>245</v>
-      </c>
-      <c r="E66" t="s">
-        <v>129</v>
+        <v>241</v>
+      </c>
+      <c r="G66">
+        <v>107</v>
       </c>
       <c r="H66" s="1">
-        <v>46257</v>
+        <v>46199</v>
+      </c>
+      <c r="I66" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="J66" s="3" t="s">
+        <v>397</v>
       </c>
       <c r="K66" t="s">
         <v>196</v>
       </c>
       <c r="M66" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="N66" t="s">
-        <v>125</v>
+        <v>20</v>
+      </c>
+      <c r="O66" t="s">
+        <v>297</v>
       </c>
       <c r="P66" t="s">
-        <v>355</v>
+        <v>319</v>
       </c>
       <c r="Q66" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="R66" t="s">
-        <v>127</v>
+        <v>22</v>
       </c>
     </row>
     <row r="67" spans="1:18" x14ac:dyDescent="0.45">
@@ -7190,7 +7199,7 @@
     </sortState>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="M43" r:id="rId1" xr:uid="{5644AB62-A977-428F-9FE2-4F7F37CACBD0}"/>
+    <hyperlink ref="M44" r:id="rId1" xr:uid="{5644AB62-A977-428F-9FE2-4F7F37CACBD0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Timeline order fix DCU
</commit_message>
<xml_diff>
--- a/DCU.xlsx
+++ b/DCU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{709161FB-D2AA-44F0-BDE9-14EE3B334AEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00905BDB-DB2F-4CEC-B971-07665059CBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2550,7 +2550,7 @@
         <v>66</v>
       </c>
       <c r="C21">
-        <v>66</v>
+        <v>20</v>
       </c>
       <c r="D21" t="s">
         <v>245</v>
@@ -2600,7 +2600,7 @@
         <v>64</v>
       </c>
       <c r="C22">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D22" t="s">
         <v>245</v>
@@ -2650,7 +2650,7 @@
         <v>65</v>
       </c>
       <c r="C23">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="D23" t="s">
         <v>245</v>
@@ -2700,7 +2700,7 @@
         <v>17</v>
       </c>
       <c r="C24">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D24" t="s">
         <v>100</v>
@@ -2747,7 +2747,7 @@
         <v>18</v>
       </c>
       <c r="C25">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D25" t="s">
         <v>104</v>
@@ -2794,7 +2794,7 @@
         <v>19</v>
       </c>
       <c r="C26">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D26" t="s">
         <v>108</v>
@@ -2841,7 +2841,7 @@
         <v>21</v>
       </c>
       <c r="C27">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D27" t="s">
         <v>112</v>
@@ -2888,7 +2888,7 @@
         <v>23</v>
       </c>
       <c r="C28">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D28" t="s">
         <v>116</v>
@@ -2935,7 +2935,7 @@
         <v>24</v>
       </c>
       <c r="C29">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D29" t="s">
         <v>121</v>
@@ -2985,7 +2985,7 @@
         <v>25</v>
       </c>
       <c r="C30">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D30" t="s">
         <v>121</v>
@@ -3035,7 +3035,7 @@
         <v>26</v>
       </c>
       <c r="C31">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D31" t="s">
         <v>121</v>
@@ -3085,7 +3085,7 @@
         <v>27</v>
       </c>
       <c r="C32">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D32" t="s">
         <v>121</v>
@@ -3135,7 +3135,7 @@
         <v>28</v>
       </c>
       <c r="C33">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D33" t="s">
         <v>121</v>
@@ -3185,7 +3185,7 @@
         <v>29</v>
       </c>
       <c r="C34">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D34" t="s">
         <v>121</v>
@@ -3235,7 +3235,7 @@
         <v>30</v>
       </c>
       <c r="C35">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D35" t="s">
         <v>121</v>
@@ -3285,7 +3285,7 @@
         <v>31</v>
       </c>
       <c r="C36">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D36" t="s">
         <v>121</v>
@@ -3335,7 +3335,7 @@
         <v>33</v>
       </c>
       <c r="C37">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D37" t="s">
         <v>150</v>
@@ -3379,7 +3379,7 @@
         <v>34</v>
       </c>
       <c r="C38">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D38" t="s">
         <v>154</v>
@@ -3423,7 +3423,7 @@
         <v>35</v>
       </c>
       <c r="C39">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D39" t="s">
         <v>158</v>
@@ -3467,7 +3467,7 @@
         <v>32</v>
       </c>
       <c r="C40">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D40" t="s">
         <v>162</v>
@@ -3511,7 +3511,7 @@
         <v>38</v>
       </c>
       <c r="C41">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D41" t="s">
         <v>167</v>
@@ -3558,7 +3558,7 @@
         <v>39</v>
       </c>
       <c r="C42">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D42" t="s">
         <v>167</v>
@@ -3605,7 +3605,7 @@
         <v>41</v>
       </c>
       <c r="C43">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D43" t="s">
         <v>167</v>
@@ -3652,7 +3652,7 @@
         <v>42</v>
       </c>
       <c r="C44">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D44" t="s">
         <v>167</v>
@@ -3699,7 +3699,7 @@
         <v>43</v>
       </c>
       <c r="C45">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D45" t="s">
         <v>167</v>
@@ -3746,7 +3746,7 @@
         <v>44</v>
       </c>
       <c r="C46">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D46" t="s">
         <v>167</v>
@@ -3793,7 +3793,7 @@
         <v>45</v>
       </c>
       <c r="C47">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D47" t="s">
         <v>167</v>
@@ -3840,7 +3840,7 @@
         <v>46</v>
       </c>
       <c r="C48">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D48" t="s">
         <v>167</v>
@@ -3887,7 +3887,7 @@
         <v>37</v>
       </c>
       <c r="C49">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D49" t="s">
         <v>186</v>
@@ -3931,7 +3931,7 @@
         <v>36</v>
       </c>
       <c r="C50">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D50" t="s">
         <v>190</v>
@@ -3975,7 +3975,7 @@
         <v>47</v>
       </c>
       <c r="C51">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D51" t="s">
         <v>194</v>
@@ -4025,7 +4025,7 @@
         <v>48</v>
       </c>
       <c r="C52">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D52" t="s">
         <v>194</v>
@@ -4075,7 +4075,7 @@
         <v>49</v>
       </c>
       <c r="C53">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D53" t="s">
         <v>194</v>
@@ -4125,7 +4125,7 @@
         <v>50</v>
       </c>
       <c r="C54">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D54" t="s">
         <v>194</v>
@@ -4175,7 +4175,7 @@
         <v>51</v>
       </c>
       <c r="C55">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D55" t="s">
         <v>194</v>
@@ -4225,7 +4225,7 @@
         <v>52</v>
       </c>
       <c r="C56">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D56" t="s">
         <v>194</v>
@@ -4275,7 +4275,7 @@
         <v>53</v>
       </c>
       <c r="C57">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D57" t="s">
         <v>194</v>
@@ -4325,7 +4325,7 @@
         <v>54</v>
       </c>
       <c r="C58">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D58" t="s">
         <v>29</v>
@@ -4372,7 +4372,7 @@
         <v>55</v>
       </c>
       <c r="C59">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D59" t="s">
         <v>121</v>
@@ -4422,7 +4422,7 @@
         <v>56</v>
       </c>
       <c r="C60">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D60" t="s">
         <v>121</v>
@@ -4472,7 +4472,7 @@
         <v>57</v>
       </c>
       <c r="C61">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D61" t="s">
         <v>121</v>
@@ -4522,7 +4522,7 @@
         <v>58</v>
       </c>
       <c r="C62">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D62" t="s">
         <v>121</v>
@@ -4572,7 +4572,7 @@
         <v>59</v>
       </c>
       <c r="C63">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D63" t="s">
         <v>121</v>
@@ -4622,7 +4622,7 @@
         <v>60</v>
       </c>
       <c r="C64">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D64" t="s">
         <v>121</v>
@@ -4672,7 +4672,7 @@
         <v>61</v>
       </c>
       <c r="C65">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D65" t="s">
         <v>121</v>
@@ -4722,7 +4722,7 @@
         <v>62</v>
       </c>
       <c r="C66">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D66" t="s">
         <v>121</v>
@@ -4772,7 +4772,7 @@
         <v>63</v>
       </c>
       <c r="C67">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D67" t="s">
         <v>241</v>

</xml_diff>